<commit_message>
feat(battle): configure STS starter deck
</commit_message>
<xml_diff>
--- a/DataTables/Datas/__enums__.xlsx
+++ b/DataTables/Datas/__enums__.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{920E6008-DAFB-4B41-A9B3-A4D4311CA86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC6DBF38-4CB6-4E9C-8E65-AF94C55A3352}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9060" yWindow="5535" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="5535" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
   <si>
     <t>##var</t>
   </si>
@@ -82,16 +82,28 @@
     <t>battle.TargetRule</t>
   </si>
   <si>
+    <t>Self target only</t>
+  </si>
+  <si>
+    <t>battle.EffectType</t>
+  </si>
+  <si>
+    <t>Modify an attribute</t>
+  </si>
+  <si>
+    <t>battle.Attribute</t>
+  </si>
+  <si>
+    <t>Strength</t>
+  </si>
+  <si>
     <t>Card target rule</t>
   </si>
   <si>
     <t>Self</t>
   </si>
   <si>
-    <t>Self target only</t>
-  </si>
-  <si>
-    <t>battle.EffectType</t>
+    <t>Enemy</t>
   </si>
   <si>
     <t>Card effect type</t>
@@ -100,16 +112,19 @@
     <t>ModifyAttribute</t>
   </si>
   <si>
-    <t>Modify an attribute</t>
-  </si>
-  <si>
-    <t>battle.Attribute</t>
+    <t>DealDamage</t>
+  </si>
+  <si>
+    <t>GainBlock</t>
+  </si>
+  <si>
+    <t>ApplyVulnerable</t>
   </si>
   <si>
     <t>Attribute modifiable by card effect</t>
   </si>
   <si>
-    <t>Strength</t>
+    <t>None</t>
   </si>
 </sst>
 </file>
@@ -462,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
@@ -573,44 +588,32 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4" t="s">
         <v>20</v>
       </c>
-      <c r="H4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4" t="s">
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D5" t="b">
-        <v>1</v>
-      </c>
-      <c r="F5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5" t="s">
-        <v>25</v>
-      </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C6" t="b">
         <v>0</v>
@@ -628,7 +631,59 @@
         <v>0</v>
       </c>
       <c r="K6" t="s">
-        <v>29</v>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H7" t="s">
+        <v>30</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H8" t="s">
+        <v>31</v>
+      </c>
+      <c r="J8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H9" t="s">
+        <v>32</v>
+      </c>
+      <c r="J9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>33</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H11" t="s">
+        <v>24</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(run): complete G4 deck rewards and upgrades
</commit_message>
<xml_diff>
--- a/DataTables/Datas/__enums__.xlsx
+++ b/DataTables/Datas/__enums__.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rc13f6790b5de4446"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rfe1e9fad382e4277"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3159,6 +3159,122 @@
       </x:c>
       <x:c r="L125"/>
     </x:row>
+    <x:row r="126">
+      <x:c r="A126"/>
+      <x:c r="B126" t="str">
+        <x:v>battle.CardUpgradeTrackKind</x:v>
+      </x:c>
+      <x:c r="C126" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="D126" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="E126"/>
+      <x:c r="F126" t="str">
+        <x:v>Card upgrade track kind</x:v>
+      </x:c>
+      <x:c r="G126"/>
+      <x:c r="H126" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I126"/>
+      <x:c r="J126" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K126" t="str">
+        <x:v>No G4 upgrade track</x:v>
+      </x:c>
+      <x:c r="L126"/>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127"/>
+      <x:c r="B127"/>
+      <x:c r="C127"/>
+      <x:c r="D127"/>
+      <x:c r="E127"/>
+      <x:c r="F127"/>
+      <x:c r="G127"/>
+      <x:c r="H127" t="str">
+        <x:v>Finite</x:v>
+      </x:c>
+      <x:c r="I127"/>
+      <x:c r="J127" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K127" t="str">
+        <x:v>Explicit sequential levels</x:v>
+      </x:c>
+      <x:c r="L127"/>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128"/>
+      <x:c r="B128"/>
+      <x:c r="C128"/>
+      <x:c r="D128"/>
+      <x:c r="E128"/>
+      <x:c r="F128"/>
+      <x:c r="G128"/>
+      <x:c r="H128" t="str">
+        <x:v>Infinite</x:v>
+      </x:c>
+      <x:c r="I128"/>
+      <x:c r="J128" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K128" t="str">
+        <x:v>Typed fixed delta per level</x:v>
+      </x:c>
+      <x:c r="L128"/>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129"/>
+      <x:c r="B129" t="str">
+        <x:v>battle.CardUpgradeRuleKind</x:v>
+      </x:c>
+      <x:c r="C129" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="D129" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="E129"/>
+      <x:c r="F129" t="str">
+        <x:v>Typed card upgrade rule kind</x:v>
+      </x:c>
+      <x:c r="G129"/>
+      <x:c r="H129" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I129"/>
+      <x:c r="J129" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K129" t="str">
+        <x:v>No numeric upgrade rule</x:v>
+      </x:c>
+      <x:c r="L129"/>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130"/>
+      <x:c r="B130"/>
+      <x:c r="C130"/>
+      <x:c r="D130"/>
+      <x:c r="E130"/>
+      <x:c r="F130"/>
+      <x:c r="G130"/>
+      <x:c r="H130" t="str">
+        <x:v>DamageValue</x:v>
+      </x:c>
+      <x:c r="I130"/>
+      <x:c r="J130" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K130" t="str">
+        <x:v>Replace or add card damage value</x:v>
+      </x:c>
+      <x:c r="L130"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="H1:L1"/>

</xml_diff>